<commit_message>
[Codex] feat: standardize skill VFX sizes and redesign thrust
</commit_message>
<xml_diff>
--- a/config/Excel/Skills2.xlsx
+++ b/config/Excel/Skills2.xlsx
@@ -298,6 +298,16 @@
           <t xml:space="preserve">進一步強化突刺傷害，額外 +{pct}% 物理傷害（與第 1 階累加）</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">slash-thrust-empowered</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hit-phys</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -357,7 +367,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">slash-thrust-lance</t>
+          <t xml:space="preserve">slash-thrust-empowered</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -422,6 +432,11 @@
           <t xml:space="preserve">突刺造成的傷害有 {pct}% 會擴散至周圍的 {count} 個敵人</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">slash-thrust-scatter</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr">
         <is>
           <t xml:space="preserve">hit-phys</t>
@@ -486,7 +501,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t xml:space="preserve">slash-thrust-lance</t>
+          <t xml:space="preserve">slash-thrust-scatter</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -553,7 +568,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t xml:space="preserve">slash-thrust-lance</t>
+          <t xml:space="preserve">slash-thrust-scatter</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -13468,6 +13483,11 @@
       <c r="O231" t="inlineStr">
         <is>
           <t xml:space="preserve">施放暴風屏障時同時打出【暴風真空刃】與【虛空斬】，且這兩者的傷害額外 +{pct}%</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">burst-wind</t>
         </is>
       </c>
       <c r="R231" t="inlineStr">

</xml_diff>

<commit_message>
[Codex] feat: redesign cleave crescent and directional flight
</commit_message>
<xml_diff>
--- a/config/Excel/Skills2.xlsx
+++ b/config/Excel/Skills2.xlsx
@@ -963,6 +963,11 @@
           <t xml:space="preserve">斬擊時有 {chance}% 機率擊暈敵人 {sec} 秒</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">slash-cleave-stun</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1017,7 +1022,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t xml:space="preserve">slash-cleave-arc</t>
+          <t xml:space="preserve">slash-cleave-stun</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -1079,7 +1084,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t xml:space="preserve">slash-cleave-sector</t>
+          <t xml:space="preserve">slash-cleave-stun</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">

</xml_diff>

<commit_message>
feat(vfx): integrate counter ripple projectile and configuration changes
</commit_message>
<xml_diff>
--- a/config/Excel/Skills2.xlsx
+++ b/config/Excel/Skills2.xlsx
@@ -6737,8 +6737,10 @@
       <c r="X62" s="1">
         <v>5</v>
       </c>
-      <c r="Z62" t="s">
-        <v>274</v>
+      <c r="AA62" t="inlineStr">
+        <is>
+          <t>proj-counter-ripple</t>
+        </is>
       </c>
       <c r="AB62" t="s">
         <v>40</v>

</xml_diff>